<commit_message>
chore(data): archive validated experiment outputs
</commit_message>
<xml_diff>
--- a/output/excel/joint_gap_metrics_joint_gap_c6_u30_k3_s4_seed42.xlsx
+++ b/output/excel/joint_gap_metrics_joint_gap_c6_u30_k3_s4_seed42.xlsx
@@ -544,7 +544,7 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>26.027467</v>
+        <v>38.1272811</v>
       </c>
       <c r="M2">
         <v>26620</v>
@@ -588,7 +588,7 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <v>4.662999599999996</v>
+        <v>7.646138300000004</v>
       </c>
       <c r="M3">
         <v>8</v>
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>5.581700457362258</v>
+        <v>4.986475473507977</v>
       </c>
       <c r="F2">
         <v>327.1769010551288</v>

</xml_diff>